<commit_message>
Add Sectors API client + normalization layer for companies, reports, prices, financials, news
Typed wrappers over E-01 (companies screener), E-02 (company report),
E-03 (daily transaction), E-05 (quarterly financials), E-06/E-07 (helper
lists), and E-04 (news), each normalizing raw API responses into domain
types and stamping fetchedAt per ADD-SH2026-003 section 4. Verified
against live API; credit usage logged in the data dictionary.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Roadmap Solo Sectors Hackathon.xlsx
+++ b/docs/Roadmap Solo Sectors Hackathon.xlsx
@@ -1356,7 +1356,7 @@
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G19" s="19" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G20" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Log actual dev velocity vs roadmap estimates, reconcile credits with dashboard
Roadmap: added a velocity-notes section derived from git commit
timestamps -- 4h41m real time covered ~227 of 336 estimated roadmap
hours (68%), a ~48x compression attributable to AI-assisted development,
not a flaw in the original estimates (which remain realistic for
unassisted solo manual coding).

API Data Dictionary: final credit reconciliation against the real
Sectors dashboard (Plans & Usage) -- 195 requests used, 805 remaining,
expires Sep 30 2026. Flagged that prior manual log entries undercounted
significantly (~58 tracked vs 195 actual) and should not be trusted over
the dashboard figure.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Roadmap Solo Sectors Hackathon.xlsx
+++ b/docs/Roadmap Solo Sectors Hackathon.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AH88"/>
+  <dimension ref="A1:AH96"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4813,6 +4813,100 @@
       <c r="A88" s="4" t="inlineStr">
         <is>
           <t>Perbarui kolom Status ke Backlog / In Progress / Done / On Hold / Won't Do / Potential Delay. Kolom Jam Tersisa menunjukkan sisa beban sebenarnya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>CATATAN KECEPATAN AKTUAL (diisi 4 September 2026, berbasis timestamp commit git)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Waktu nyata untuk task 7 s/d 30 (fondasi s/d F-08 + grafik)</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>4 jam 41 menit</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Diukur dari commit pertama (16:55) sampai commit terakhir sesi (21:36)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Estimasi roadmap untuk task yang sama</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>227 jam</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>68% dari total 336 jam roadmap</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Rasio kompresi</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>~48x</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Karena bantuan AI pair-programming, bukan indikasi estimasi awal salah</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Catatan penting</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Estimasi 12,5 jam/hari x 27 hari REALISTIS untuk solo coding manual tanpa AI. Kompresi terjadi karena mode kerja berbeda (AI-assisted), bukan karena estimasi awal keliru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Yang TIDAK ikut terkompresi</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Waktu tunggu API eksternal (mis. gangguan Gemini 503 memakan puluhan menit), video/narasi (kerja kreatif manusia), review manual/QA akhir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Implikasi</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Sisa task dev (tooltip, bug fixing, polish) realistis selesai dalam hitungan jam-hari, bukan minggu. Sisa waktu (26 hari ke deadline 30 Sep) dialokasikan ke: testing lebih dalam, video/narasi matang, buffer risiko.</t>
         </is>
       </c>
     </row>

</xml_diff>